<commit_message>
feat: Opp1 = niveau de diplôme communal INSEE (18 ans et plus), en remplacement d'une suite artificielle
Opp1.xlsx contenait un compteur (5,75 ; 5,76 ...) sans rapport avec l'éducation. Opp1 est maintenant calculé
depuis le recensement INSEE 2020 (base IRIS Diplômes-Formation, 15-17 ans non scolarisés retirés), puis scores,
seuils de Jenks, LISA, CAH, classement Excel et documentation sont régénérés. Les scripts CAH lisaient un
GeoJSON inexistant dans le dépôt : chemin corrigé.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/stats_descriptives_betti_0_10.xlsx
+++ b/downloads/stats_descriptives_betti_0_10.xlsx
@@ -503,37 +503,37 @@
         <v>360</v>
       </c>
       <c r="C2" t="n">
-        <v>3.362216</v>
+        <v>4.080344</v>
       </c>
       <c r="D2" t="n">
-        <v>1.358776</v>
+        <v>1.497156</v>
       </c>
       <c r="E2" t="n">
-        <v>1.846273</v>
+        <v>2.241476</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>2.501941</v>
+        <v>3.128716</v>
       </c>
       <c r="H2" t="n">
-        <v>3.125731</v>
+        <v>3.951261</v>
       </c>
       <c r="I2" t="n">
-        <v>3.991717</v>
+        <v>4.748026</v>
       </c>
       <c r="J2" t="n">
         <v>10</v>
       </c>
       <c r="K2" t="n">
-        <v>1.489776</v>
+        <v>1.61931</v>
       </c>
       <c r="L2" t="n">
-        <v>2.501941</v>
+        <v>3.128716</v>
       </c>
       <c r="M2" t="n">
-        <v>3.991717</v>
+        <v>4.748026</v>
       </c>
     </row>
     <row r="3">
@@ -546,37 +546,37 @@
         <v>360</v>
       </c>
       <c r="C3" t="n">
-        <v>0.06936199999999999</v>
+        <v>0.089048</v>
       </c>
       <c r="D3" t="n">
-        <v>0.018764</v>
+        <v>0.020546</v>
       </c>
       <c r="E3" t="n">
-        <v>0.000352</v>
+        <v>0.000422</v>
       </c>
       <c r="F3" t="n">
-        <v>0.022931</v>
+        <v>0.033052</v>
       </c>
       <c r="G3" t="n">
-        <v>0.057482</v>
+        <v>0.075988</v>
       </c>
       <c r="H3" t="n">
-        <v>0.066096</v>
+        <v>0.08727600000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>0.078055</v>
+        <v>0.09821100000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>0.161027</v>
+        <v>0.170284</v>
       </c>
       <c r="K3" t="n">
-        <v>0.020573</v>
+        <v>0.022222</v>
       </c>
       <c r="L3" t="n">
-        <v>0.057482</v>
+        <v>0.075988</v>
       </c>
       <c r="M3" t="n">
-        <v>0.078055</v>
+        <v>0.09821100000000001</v>
       </c>
     </row>
     <row r="4">
@@ -589,37 +589,37 @@
         <v>360</v>
       </c>
       <c r="C4" t="n">
-        <v>3.874089</v>
+        <v>4.847696</v>
       </c>
       <c r="D4" t="n">
-        <v>1.583946</v>
+        <v>1.790199</v>
       </c>
       <c r="E4" t="n">
-        <v>2.508885</v>
+        <v>3.204812</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>2.742758</v>
+        <v>3.580625</v>
       </c>
       <c r="H4" t="n">
-        <v>3.757793</v>
+        <v>4.884653</v>
       </c>
       <c r="I4" t="n">
-        <v>4.816753</v>
+        <v>6.089257</v>
       </c>
       <c r="J4" t="n">
         <v>10</v>
       </c>
       <c r="K4" t="n">
-        <v>2.073996</v>
+        <v>2.508632</v>
       </c>
       <c r="L4" t="n">
-        <v>2.742758</v>
+        <v>3.580625</v>
       </c>
       <c r="M4" t="n">
-        <v>4.816753</v>
+        <v>6.089257</v>
       </c>
     </row>
     <row r="5">
@@ -632,37 +632,37 @@
         <v>360</v>
       </c>
       <c r="C5" t="n">
-        <v>0.346565</v>
+        <v>0.424299</v>
       </c>
       <c r="D5" t="n">
-        <v>0.093843</v>
+        <v>0.08806</v>
       </c>
       <c r="E5" t="n">
-        <v>0.008807000000000001</v>
+        <v>0.007755</v>
       </c>
       <c r="F5" t="n">
-        <v>0.117039</v>
+        <v>0.185841</v>
       </c>
       <c r="G5" t="n">
-        <v>0.279538</v>
+        <v>0.361972</v>
       </c>
       <c r="H5" t="n">
-        <v>0.339675</v>
+        <v>0.426117</v>
       </c>
       <c r="I5" t="n">
-        <v>0.402415</v>
+        <v>0.485372</v>
       </c>
       <c r="J5" t="n">
-        <v>0.709504</v>
+        <v>0.677741</v>
       </c>
       <c r="K5" t="n">
-        <v>0.122877</v>
+        <v>0.1234</v>
       </c>
       <c r="L5" t="n">
-        <v>0.279538</v>
+        <v>0.361972</v>
       </c>
       <c r="M5" t="n">
-        <v>0.402415</v>
+        <v>0.485372</v>
       </c>
     </row>
     <row r="6">
@@ -923,37 +923,37 @@
         <v>360</v>
       </c>
       <c r="C2" t="n">
-        <v>3.874089</v>
+        <v>4.847696</v>
       </c>
       <c r="D2" t="n">
-        <v>1.583946</v>
+        <v>1.790199</v>
       </c>
       <c r="E2" t="n">
-        <v>2.508885</v>
+        <v>3.204812</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>2.742758</v>
+        <v>3.580625</v>
       </c>
       <c r="H2" t="n">
-        <v>3.757793</v>
+        <v>4.884653</v>
       </c>
       <c r="I2" t="n">
-        <v>4.816753</v>
+        <v>6.089257</v>
       </c>
       <c r="J2" t="n">
         <v>10</v>
       </c>
       <c r="K2" t="n">
-        <v>2.073996</v>
+        <v>2.508632</v>
       </c>
       <c r="L2" t="n">
-        <v>2.742758</v>
+        <v>3.580625</v>
       </c>
       <c r="M2" t="n">
-        <v>4.816753</v>
+        <v>6.089257</v>
       </c>
     </row>
     <row r="3">
@@ -966,37 +966,37 @@
         <v>360</v>
       </c>
       <c r="C3" t="n">
-        <v>0.346565</v>
+        <v>0.424299</v>
       </c>
       <c r="D3" t="n">
-        <v>0.093843</v>
+        <v>0.08806</v>
       </c>
       <c r="E3" t="n">
-        <v>0.008807000000000001</v>
+        <v>0.007755</v>
       </c>
       <c r="F3" t="n">
-        <v>0.117039</v>
+        <v>0.185841</v>
       </c>
       <c r="G3" t="n">
-        <v>0.279538</v>
+        <v>0.361972</v>
       </c>
       <c r="H3" t="n">
-        <v>0.339675</v>
+        <v>0.426117</v>
       </c>
       <c r="I3" t="n">
-        <v>0.402415</v>
+        <v>0.485372</v>
       </c>
       <c r="J3" t="n">
-        <v>0.709504</v>
+        <v>0.677741</v>
       </c>
       <c r="K3" t="n">
-        <v>0.122877</v>
+        <v>0.1234</v>
       </c>
       <c r="L3" t="n">
-        <v>0.279538</v>
+        <v>0.361972</v>
       </c>
       <c r="M3" t="n">
-        <v>0.402415</v>
+        <v>0.485372</v>
       </c>
     </row>
     <row r="4">
@@ -1009,37 +1009,37 @@
         <v>360</v>
       </c>
       <c r="C4" t="n">
-        <v>5.308875</v>
+        <v>3.402056</v>
       </c>
       <c r="D4" t="n">
-        <v>0.180446</v>
+        <v>0.398355</v>
       </c>
       <c r="E4" t="n">
-        <v>0.032561</v>
+        <v>0.158687</v>
       </c>
       <c r="F4" t="n">
-        <v>5.1</v>
+        <v>2</v>
       </c>
       <c r="G4" t="n">
-        <v>5.18975</v>
+        <v>3.117641</v>
       </c>
       <c r="H4" t="n">
-        <v>5.2795</v>
+        <v>3.393121</v>
       </c>
       <c r="I4" t="n">
-        <v>5.36925</v>
+        <v>3.681762</v>
       </c>
       <c r="J4" t="n">
-        <v>5.99</v>
+        <v>4.56962</v>
       </c>
       <c r="K4" t="n">
-        <v>0.1795</v>
+        <v>0.564121</v>
       </c>
       <c r="L4" t="n">
-        <v>5.18975</v>
+        <v>3.117641</v>
       </c>
       <c r="M4" t="n">
-        <v>5.36925</v>
+        <v>3.681762</v>
       </c>
     </row>
     <row r="5">
@@ -1052,37 +1052,37 @@
         <v>360</v>
       </c>
       <c r="C5" t="n">
-        <v>2.34691</v>
+        <v>5.456277</v>
       </c>
       <c r="D5" t="n">
-        <v>2.027484</v>
+        <v>1.55025</v>
       </c>
       <c r="E5" t="n">
-        <v>4.11069</v>
+        <v>2.403276</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>1.008427</v>
+        <v>4.349439</v>
       </c>
       <c r="H5" t="n">
-        <v>2.016854</v>
+        <v>5.421506</v>
       </c>
       <c r="I5" t="n">
-        <v>3.025281</v>
+        <v>6.544787</v>
       </c>
       <c r="J5" t="n">
         <v>10</v>
       </c>
       <c r="K5" t="n">
-        <v>2.016854</v>
+        <v>2.195348</v>
       </c>
       <c r="L5" t="n">
-        <v>1.008427</v>
+        <v>4.349439</v>
       </c>
       <c r="M5" t="n">
-        <v>3.025281</v>
+        <v>6.544787</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
feat: indice courant v2 — sources officielles de millésime homogène (recensement 2023, ARCEP T4 2024, IRCOM revenus 2024, QPV 2024, BPE 2024)
- construire_indice_v2.py : 10 indicateurs commune par commune, composantes et provenance dans Données/indice_v2/sources_indice_v2.json ; extraire_corse_xlsx.py pour les bases INSEE 2023
- Vec1 = revenu fiscal moyen par foyer (IRCOM) ; Opp4 recalculé depuis l'ARCEP (4G au moins un opérateur) ; Cho1 = population officielle des QPV ; Vec2 sans terme de confort ; Vec3 à 3 catégories
- exporter_sous_composantes.py et regenerer_data_scores.py lisent la v2 ; Jenks, LISA, CAH, chatbot, Excel, EPCI régénérés ; variante Vec1 retirée (archivée)
- ancien indice archivé (Données/archive_indice_v1_2020_2024, étiquette indice-courant-v1-2020-2024) ; série Évolution alignée sur Vec2 et Vec3 ; tests et documentation mis à jour

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/stats_descriptives_betti_0_10.xlsx
+++ b/downloads/stats_descriptives_betti_0_10.xlsx
@@ -503,37 +503,37 @@
         <v>360</v>
       </c>
       <c r="C2" t="n">
-        <v>4.080344</v>
+        <v>4.280791</v>
       </c>
       <c r="D2" t="n">
-        <v>1.497156</v>
+        <v>1.884743</v>
       </c>
       <c r="E2" t="n">
-        <v>2.241476</v>
+        <v>3.552256</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>3.128716</v>
+        <v>2.947068</v>
       </c>
       <c r="H2" t="n">
-        <v>3.951261</v>
+        <v>4.226464</v>
       </c>
       <c r="I2" t="n">
-        <v>4.748026</v>
+        <v>5.402328</v>
       </c>
       <c r="J2" t="n">
         <v>10</v>
       </c>
       <c r="K2" t="n">
-        <v>1.61931</v>
+        <v>2.45526</v>
       </c>
       <c r="L2" t="n">
-        <v>3.128716</v>
+        <v>2.947068</v>
       </c>
       <c r="M2" t="n">
-        <v>4.748026</v>
+        <v>5.402328</v>
       </c>
     </row>
     <row r="3">
@@ -546,37 +546,37 @@
         <v>360</v>
       </c>
       <c r="C3" t="n">
-        <v>0.089048</v>
+        <v>0.07385700000000001</v>
       </c>
       <c r="D3" t="n">
-        <v>0.020546</v>
+        <v>0.0214</v>
       </c>
       <c r="E3" t="n">
-        <v>0.000422</v>
+        <v>0.000458</v>
       </c>
       <c r="F3" t="n">
-        <v>0.033052</v>
+        <v>0.025252</v>
       </c>
       <c r="G3" t="n">
-        <v>0.075988</v>
+        <v>0.058713</v>
       </c>
       <c r="H3" t="n">
-        <v>0.08727600000000001</v>
+        <v>0.07324</v>
       </c>
       <c r="I3" t="n">
-        <v>0.09821100000000001</v>
+        <v>0.086591</v>
       </c>
       <c r="J3" t="n">
-        <v>0.170284</v>
+        <v>0.138794</v>
       </c>
       <c r="K3" t="n">
-        <v>0.022222</v>
+        <v>0.027878</v>
       </c>
       <c r="L3" t="n">
-        <v>0.075988</v>
+        <v>0.058713</v>
       </c>
       <c r="M3" t="n">
-        <v>0.09821100000000001</v>
+        <v>0.086591</v>
       </c>
     </row>
     <row r="4">
@@ -589,37 +589,37 @@
         <v>360</v>
       </c>
       <c r="C4" t="n">
-        <v>4.847696</v>
+        <v>5.638079</v>
       </c>
       <c r="D4" t="n">
-        <v>1.790199</v>
+        <v>2.104138</v>
       </c>
       <c r="E4" t="n">
-        <v>3.204812</v>
+        <v>4.427398</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>3.580625</v>
+        <v>4.028159</v>
       </c>
       <c r="H4" t="n">
-        <v>4.884653</v>
+        <v>5.968596</v>
       </c>
       <c r="I4" t="n">
-        <v>6.089257</v>
+        <v>7.419413</v>
       </c>
       <c r="J4" t="n">
         <v>10</v>
       </c>
       <c r="K4" t="n">
-        <v>2.508632</v>
+        <v>3.391255</v>
       </c>
       <c r="L4" t="n">
-        <v>3.580625</v>
+        <v>4.028159</v>
       </c>
       <c r="M4" t="n">
-        <v>6.089257</v>
+        <v>7.419413</v>
       </c>
     </row>
     <row r="5">
@@ -632,37 +632,37 @@
         <v>360</v>
       </c>
       <c r="C5" t="n">
-        <v>0.424299</v>
+        <v>0.424992</v>
       </c>
       <c r="D5" t="n">
-        <v>0.08806</v>
+        <v>0.122292</v>
       </c>
       <c r="E5" t="n">
-        <v>0.007755</v>
+        <v>0.014955</v>
       </c>
       <c r="F5" t="n">
-        <v>0.185841</v>
+        <v>0.09730900000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>0.361972</v>
+        <v>0.331424</v>
       </c>
       <c r="H5" t="n">
-        <v>0.426117</v>
+        <v>0.444201</v>
       </c>
       <c r="I5" t="n">
-        <v>0.485372</v>
+        <v>0.528522</v>
       </c>
       <c r="J5" t="n">
-        <v>0.677741</v>
+        <v>0.678505</v>
       </c>
       <c r="K5" t="n">
-        <v>0.1234</v>
+        <v>0.197098</v>
       </c>
       <c r="L5" t="n">
-        <v>0.361972</v>
+        <v>0.331424</v>
       </c>
       <c r="M5" t="n">
-        <v>0.485372</v>
+        <v>0.528522</v>
       </c>
     </row>
     <row r="6">
@@ -675,37 +675,37 @@
         <v>360</v>
       </c>
       <c r="C6" t="n">
-        <v>8.793184</v>
+        <v>8.833892000000001</v>
       </c>
       <c r="D6" t="n">
-        <v>1.422896</v>
+        <v>1.367206</v>
       </c>
       <c r="E6" t="n">
-        <v>2.024632</v>
+        <v>1.869253</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>8.552103000000001</v>
+        <v>8.564321</v>
       </c>
       <c r="H6" t="n">
-        <v>9.199036</v>
+        <v>9.206726</v>
       </c>
       <c r="I6" t="n">
-        <v>9.595499999999999</v>
+        <v>9.605924999999999</v>
       </c>
       <c r="J6" t="n">
         <v>10</v>
       </c>
       <c r="K6" t="n">
-        <v>1.043397</v>
+        <v>1.041604</v>
       </c>
       <c r="L6" t="n">
-        <v>8.552103000000001</v>
+        <v>8.564321</v>
       </c>
       <c r="M6" t="n">
-        <v>9.595499999999999</v>
+        <v>9.605924999999999</v>
       </c>
     </row>
     <row r="7">
@@ -718,37 +718,37 @@
         <v>360</v>
       </c>
       <c r="C7" t="n">
-        <v>0.921158</v>
+        <v>0.922834</v>
       </c>
       <c r="D7" t="n">
-        <v>0.092959</v>
+        <v>0.090473</v>
       </c>
       <c r="E7" t="n">
-        <v>0.008640999999999999</v>
+        <v>0.008185</v>
       </c>
       <c r="F7" t="n">
-        <v>0.346692</v>
+        <v>0.338263</v>
       </c>
       <c r="G7" t="n">
-        <v>0.905408</v>
+        <v>0.904996</v>
       </c>
       <c r="H7" t="n">
-        <v>0.947672</v>
+        <v>0.947506</v>
       </c>
       <c r="I7" t="n">
-        <v>0.9735740000000001</v>
+        <v>0.973923</v>
       </c>
       <c r="J7" t="n">
         <v>1</v>
       </c>
       <c r="K7" t="n">
-        <v>0.068166</v>
+        <v>0.068927</v>
       </c>
       <c r="L7" t="n">
-        <v>0.905408</v>
+        <v>0.904996</v>
       </c>
       <c r="M7" t="n">
-        <v>0.9735740000000001</v>
+        <v>0.973923</v>
       </c>
     </row>
     <row r="8">
@@ -761,37 +761,37 @@
         <v>360</v>
       </c>
       <c r="C8" t="n">
-        <v>3.46923</v>
+        <v>4.312451</v>
       </c>
       <c r="D8" t="n">
-        <v>1.445621</v>
+        <v>1.458158</v>
       </c>
       <c r="E8" t="n">
-        <v>2.08982</v>
+        <v>2.126226</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>2.695203</v>
+        <v>3.357733</v>
       </c>
       <c r="H8" t="n">
-        <v>3.414805</v>
+        <v>4.250709</v>
       </c>
       <c r="I8" t="n">
-        <v>4.173039</v>
+        <v>5.078103</v>
       </c>
       <c r="J8" t="n">
         <v>10</v>
       </c>
       <c r="K8" t="n">
-        <v>1.477836</v>
+        <v>1.72037</v>
       </c>
       <c r="L8" t="n">
-        <v>2.695203</v>
+        <v>3.357733</v>
       </c>
       <c r="M8" t="n">
-        <v>4.173039</v>
+        <v>5.078103</v>
       </c>
     </row>
     <row r="9">
@@ -804,37 +804,37 @@
         <v>360</v>
       </c>
       <c r="C9" t="n">
-        <v>0.510338</v>
+        <v>0.438089</v>
       </c>
       <c r="D9" t="n">
-        <v>0.077488</v>
+        <v>0.079605</v>
       </c>
       <c r="E9" t="n">
-        <v>0.006004</v>
+        <v>0.006337</v>
       </c>
       <c r="F9" t="n">
-        <v>0.324382</v>
+        <v>0.202659</v>
       </c>
       <c r="G9" t="n">
-        <v>0.468849</v>
+        <v>0.385968</v>
       </c>
       <c r="H9" t="n">
-        <v>0.507421</v>
+        <v>0.434719</v>
       </c>
       <c r="I9" t="n">
-        <v>0.548064</v>
+        <v>0.479889</v>
       </c>
       <c r="J9" t="n">
-        <v>0.860398</v>
+        <v>0.748591</v>
       </c>
       <c r="K9" t="n">
-        <v>0.07921400000000001</v>
+        <v>0.09392</v>
       </c>
       <c r="L9" t="n">
-        <v>0.468849</v>
+        <v>0.385968</v>
       </c>
       <c r="M9" t="n">
-        <v>0.548064</v>
+        <v>0.479889</v>
       </c>
     </row>
   </sheetData>
@@ -923,37 +923,37 @@
         <v>360</v>
       </c>
       <c r="C2" t="n">
-        <v>4.847696</v>
+        <v>5.638079</v>
       </c>
       <c r="D2" t="n">
-        <v>1.790199</v>
+        <v>2.104138</v>
       </c>
       <c r="E2" t="n">
-        <v>3.204812</v>
+        <v>4.427398</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>3.580625</v>
+        <v>4.028159</v>
       </c>
       <c r="H2" t="n">
-        <v>4.884653</v>
+        <v>5.968596</v>
       </c>
       <c r="I2" t="n">
-        <v>6.089257</v>
+        <v>7.419413</v>
       </c>
       <c r="J2" t="n">
         <v>10</v>
       </c>
       <c r="K2" t="n">
-        <v>2.508632</v>
+        <v>3.391255</v>
       </c>
       <c r="L2" t="n">
-        <v>3.580625</v>
+        <v>4.028159</v>
       </c>
       <c r="M2" t="n">
-        <v>6.089257</v>
+        <v>7.419413</v>
       </c>
     </row>
     <row r="3">
@@ -966,37 +966,37 @@
         <v>360</v>
       </c>
       <c r="C3" t="n">
-        <v>0.424299</v>
+        <v>0.424992</v>
       </c>
       <c r="D3" t="n">
-        <v>0.08806</v>
+        <v>0.122292</v>
       </c>
       <c r="E3" t="n">
-        <v>0.007755</v>
+        <v>0.014955</v>
       </c>
       <c r="F3" t="n">
-        <v>0.185841</v>
+        <v>0.09730900000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>0.361972</v>
+        <v>0.331424</v>
       </c>
       <c r="H3" t="n">
-        <v>0.426117</v>
+        <v>0.444201</v>
       </c>
       <c r="I3" t="n">
-        <v>0.485372</v>
+        <v>0.528522</v>
       </c>
       <c r="J3" t="n">
-        <v>0.677741</v>
+        <v>0.678505</v>
       </c>
       <c r="K3" t="n">
-        <v>0.1234</v>
+        <v>0.197098</v>
       </c>
       <c r="L3" t="n">
-        <v>0.361972</v>
+        <v>0.331424</v>
       </c>
       <c r="M3" t="n">
-        <v>0.485372</v>
+        <v>0.528522</v>
       </c>
     </row>
     <row r="4">
@@ -1009,37 +1009,37 @@
         <v>360</v>
       </c>
       <c r="C4" t="n">
-        <v>3.402056</v>
+        <v>3.530867</v>
       </c>
       <c r="D4" t="n">
-        <v>0.398355</v>
+        <v>0.387917</v>
       </c>
       <c r="E4" t="n">
-        <v>0.158687</v>
+        <v>0.15048</v>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>2.130435</v>
       </c>
       <c r="G4" t="n">
-        <v>3.117641</v>
+        <v>3.244799</v>
       </c>
       <c r="H4" t="n">
-        <v>3.393121</v>
+        <v>3.570369</v>
       </c>
       <c r="I4" t="n">
-        <v>3.681762</v>
+        <v>3.773379</v>
       </c>
       <c r="J4" t="n">
-        <v>4.56962</v>
+        <v>4.666667</v>
       </c>
       <c r="K4" t="n">
-        <v>0.564121</v>
+        <v>0.52858</v>
       </c>
       <c r="L4" t="n">
-        <v>3.117641</v>
+        <v>3.244799</v>
       </c>
       <c r="M4" t="n">
-        <v>3.681762</v>
+        <v>3.773379</v>
       </c>
     </row>
     <row r="5">
@@ -1052,37 +1052,37 @@
         <v>360</v>
       </c>
       <c r="C5" t="n">
-        <v>5.456277</v>
+        <v>5.521705</v>
       </c>
       <c r="D5" t="n">
-        <v>1.55025</v>
+        <v>1.529502</v>
       </c>
       <c r="E5" t="n">
-        <v>2.403276</v>
+        <v>2.339378</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>4.349439</v>
+        <v>4.393778</v>
       </c>
       <c r="H5" t="n">
-        <v>5.421506</v>
+        <v>5.677456</v>
       </c>
       <c r="I5" t="n">
-        <v>6.544787</v>
+        <v>6.477893</v>
       </c>
       <c r="J5" t="n">
         <v>10</v>
       </c>
       <c r="K5" t="n">
-        <v>2.195348</v>
+        <v>2.084114</v>
       </c>
       <c r="L5" t="n">
-        <v>4.349439</v>
+        <v>4.393778</v>
       </c>
       <c r="M5" t="n">
-        <v>6.544787</v>
+        <v>6.477893</v>
       </c>
     </row>
     <row r="6">
@@ -1095,37 +1095,37 @@
         <v>360</v>
       </c>
       <c r="C6" t="n">
-        <v>0.337934</v>
+        <v>0.389002</v>
       </c>
       <c r="D6" t="n">
-        <v>0.136854</v>
+        <v>0.19685</v>
       </c>
       <c r="E6" t="n">
-        <v>0.018729</v>
+        <v>0.03875</v>
       </c>
       <c r="F6" t="n">
-        <v>0.099479</v>
+        <v>0.120463</v>
       </c>
       <c r="G6" t="n">
-        <v>0.239636</v>
+        <v>0.259543</v>
       </c>
       <c r="H6" t="n">
-        <v>0.299413</v>
+        <v>0.335847</v>
       </c>
       <c r="I6" t="n">
-        <v>0.412237</v>
+        <v>0.47874</v>
       </c>
       <c r="J6" t="n">
-        <v>1.015732</v>
+        <v>1.436583</v>
       </c>
       <c r="K6" t="n">
-        <v>0.172601</v>
+        <v>0.219197</v>
       </c>
       <c r="L6" t="n">
-        <v>0.239636</v>
+        <v>0.259543</v>
       </c>
       <c r="M6" t="n">
-        <v>0.412237</v>
+        <v>0.47874</v>
       </c>
     </row>
     <row r="7">
@@ -1138,37 +1138,37 @@
         <v>360</v>
       </c>
       <c r="C7" t="n">
-        <v>2.6025</v>
+        <v>2.040383</v>
       </c>
       <c r="D7" t="n">
-        <v>1.493622</v>
+        <v>1.495682</v>
       </c>
       <c r="E7" t="n">
-        <v>2.230908</v>
+        <v>2.237064</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>1.529682</v>
+        <v>1.056743</v>
       </c>
       <c r="H7" t="n">
-        <v>2.182086</v>
+        <v>1.636503</v>
       </c>
       <c r="I7" t="n">
-        <v>3.413453</v>
+        <v>2.72222</v>
       </c>
       <c r="J7" t="n">
         <v>10</v>
       </c>
       <c r="K7" t="n">
-        <v>1.883771</v>
+        <v>1.665477</v>
       </c>
       <c r="L7" t="n">
-        <v>1.529682</v>
+        <v>1.056743</v>
       </c>
       <c r="M7" t="n">
-        <v>3.413453</v>
+        <v>2.72222</v>
       </c>
     </row>
     <row r="8">
@@ -1181,37 +1181,37 @@
         <v>360</v>
       </c>
       <c r="C8" t="n">
-        <v>135.698889</v>
+        <v>140.668614</v>
       </c>
       <c r="D8" t="n">
-        <v>52.681224</v>
+        <v>53.036811</v>
       </c>
       <c r="E8" t="n">
-        <v>2775.311388</v>
+        <v>2812.903366</v>
       </c>
       <c r="F8" t="n">
-        <v>62.5</v>
+        <v>63.636379</v>
       </c>
       <c r="G8" t="n">
-        <v>88.325</v>
+        <v>89.444795</v>
       </c>
       <c r="H8" t="n">
-        <v>97.95</v>
+        <v>173.055557</v>
       </c>
       <c r="I8" t="n">
-        <v>190.5</v>
+        <v>191.962104</v>
       </c>
       <c r="J8" t="n">
-        <v>294</v>
+        <v>294.288572</v>
       </c>
       <c r="K8" t="n">
-        <v>102.175</v>
+        <v>102.51731</v>
       </c>
       <c r="L8" t="n">
-        <v>88.325</v>
+        <v>89.444795</v>
       </c>
       <c r="M8" t="n">
-        <v>190.5</v>
+        <v>191.962104</v>
       </c>
     </row>
     <row r="9">
@@ -1224,37 +1224,37 @@
         <v>360</v>
       </c>
       <c r="C9" t="n">
-        <v>3.161939</v>
+        <v>3.339757</v>
       </c>
       <c r="D9" t="n">
-        <v>2.275647</v>
+        <v>2.299428</v>
       </c>
       <c r="E9" t="n">
-        <v>5.178569</v>
+        <v>5.287369</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>1.115551</v>
+        <v>1.118932</v>
       </c>
       <c r="H9" t="n">
-        <v>1.531317</v>
+        <v>4.743904</v>
       </c>
       <c r="I9" t="n">
-        <v>5.529158</v>
+        <v>5.563603</v>
       </c>
       <c r="J9" t="n">
         <v>10</v>
       </c>
       <c r="K9" t="n">
-        <v>4.413607</v>
+        <v>4.444671</v>
       </c>
       <c r="L9" t="n">
-        <v>1.115551</v>
+        <v>1.118932</v>
       </c>
       <c r="M9" t="n">
-        <v>5.529158</v>
+        <v>5.563603</v>
       </c>
     </row>
     <row r="10">
@@ -1267,37 +1267,37 @@
         <v>360</v>
       </c>
       <c r="C10" t="n">
-        <v>65.00833299999999</v>
+        <v>73.537025</v>
       </c>
       <c r="D10" t="n">
-        <v>13.966414</v>
+        <v>26.113107</v>
       </c>
       <c r="E10" t="n">
-        <v>195.060733</v>
+        <v>681.894373</v>
       </c>
       <c r="F10" t="n">
-        <v>26.666667</v>
+        <v>32.183908</v>
       </c>
       <c r="G10" t="n">
-        <v>59.666667</v>
+        <v>42.528618</v>
       </c>
       <c r="H10" t="n">
-        <v>60.166667</v>
+        <v>89.13995199999999</v>
       </c>
       <c r="I10" t="n">
-        <v>74.416667</v>
+        <v>95.19698699999999</v>
       </c>
       <c r="J10" t="n">
-        <v>93.333333</v>
+        <v>100</v>
       </c>
       <c r="K10" t="n">
-        <v>14.75</v>
+        <v>52.668369</v>
       </c>
       <c r="L10" t="n">
-        <v>59.666667</v>
+        <v>42.528618</v>
       </c>
       <c r="M10" t="n">
-        <v>74.416667</v>
+        <v>95.19698699999999</v>
       </c>
     </row>
     <row r="11">
@@ -1310,37 +1310,37 @@
         <v>360</v>
       </c>
       <c r="C11" t="n">
-        <v>5.75125</v>
+        <v>6.097833</v>
       </c>
       <c r="D11" t="n">
-        <v>2.094962</v>
+        <v>3.850577</v>
       </c>
       <c r="E11" t="n">
-        <v>4.388866</v>
+        <v>14.826942</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>4.95</v>
+        <v>1.525406</v>
       </c>
       <c r="H11" t="n">
-        <v>5.025</v>
+        <v>8.398603</v>
       </c>
       <c r="I11" t="n">
-        <v>7.1625</v>
+        <v>9.291759000000001</v>
       </c>
       <c r="J11" t="n">
         <v>10</v>
       </c>
       <c r="K11" t="n">
-        <v>2.2125</v>
+        <v>7.766353</v>
       </c>
       <c r="L11" t="n">
-        <v>4.95</v>
+        <v>1.525406</v>
       </c>
       <c r="M11" t="n">
-        <v>7.1625</v>
+        <v>9.291759000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1429,37 +1429,37 @@
         <v>360</v>
       </c>
       <c r="C2" t="n">
-        <v>8.793184</v>
+        <v>8.833892000000001</v>
       </c>
       <c r="D2" t="n">
-        <v>1.422896</v>
+        <v>1.367206</v>
       </c>
       <c r="E2" t="n">
-        <v>2.024632</v>
+        <v>1.869253</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>8.552103000000001</v>
+        <v>8.564321</v>
       </c>
       <c r="H2" t="n">
-        <v>9.199036</v>
+        <v>9.206726</v>
       </c>
       <c r="I2" t="n">
-        <v>9.595499999999999</v>
+        <v>9.605924999999999</v>
       </c>
       <c r="J2" t="n">
         <v>10</v>
       </c>
       <c r="K2" t="n">
-        <v>1.043397</v>
+        <v>1.041604</v>
       </c>
       <c r="L2" t="n">
-        <v>8.552103000000001</v>
+        <v>8.564321</v>
       </c>
       <c r="M2" t="n">
-        <v>9.595499999999999</v>
+        <v>9.605924999999999</v>
       </c>
     </row>
     <row r="3">
@@ -1472,37 +1472,37 @@
         <v>360</v>
       </c>
       <c r="C3" t="n">
-        <v>0.921158</v>
+        <v>0.922834</v>
       </c>
       <c r="D3" t="n">
-        <v>0.092959</v>
+        <v>0.090473</v>
       </c>
       <c r="E3" t="n">
-        <v>0.008640999999999999</v>
+        <v>0.008185</v>
       </c>
       <c r="F3" t="n">
-        <v>0.346692</v>
+        <v>0.338263</v>
       </c>
       <c r="G3" t="n">
-        <v>0.905408</v>
+        <v>0.904996</v>
       </c>
       <c r="H3" t="n">
-        <v>0.947672</v>
+        <v>0.947506</v>
       </c>
       <c r="I3" t="n">
-        <v>0.9735740000000001</v>
+        <v>0.973923</v>
       </c>
       <c r="J3" t="n">
         <v>1</v>
       </c>
       <c r="K3" t="n">
-        <v>0.068166</v>
+        <v>0.068927</v>
       </c>
       <c r="L3" t="n">
-        <v>0.905408</v>
+        <v>0.904996</v>
       </c>
       <c r="M3" t="n">
-        <v>0.9735740000000001</v>
+        <v>0.973923</v>
       </c>
     </row>
     <row r="4">
@@ -1515,16 +1515,16 @@
         <v>360</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.065845</v>
+        <v>-0.069437</v>
       </c>
       <c r="D4" t="n">
-        <v>0.723095</v>
+        <v>0.762516</v>
       </c>
       <c r="E4" t="n">
-        <v>0.522867</v>
+        <v>0.581431</v>
       </c>
       <c r="F4" t="n">
-        <v>-8.824237</v>
+        <v>-9.308102</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -1558,13 +1558,13 @@
         <v>360</v>
       </c>
       <c r="C5" t="n">
-        <v>9.925382000000001</v>
+        <v>9.925402</v>
       </c>
       <c r="D5" t="n">
-        <v>0.819442</v>
+        <v>0.819196</v>
       </c>
       <c r="E5" t="n">
-        <v>0.671486</v>
+        <v>0.671083</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -1601,37 +1601,37 @@
         <v>360</v>
       </c>
       <c r="C6" t="n">
-        <v>95.708139</v>
+        <v>95.80367699999999</v>
       </c>
       <c r="D6" t="n">
-        <v>4.54915</v>
+        <v>4.377765</v>
       </c>
       <c r="E6" t="n">
-        <v>20.694766</v>
+        <v>19.16483</v>
       </c>
       <c r="F6" t="n">
-        <v>71.43000000000001</v>
+        <v>71.428603</v>
       </c>
       <c r="G6" t="n">
-        <v>94.595</v>
+        <v>94.571196</v>
       </c>
       <c r="H6" t="n">
-        <v>97.01000000000001</v>
+        <v>97.000355</v>
       </c>
       <c r="I6" t="n">
-        <v>98.48999999999999</v>
+        <v>98.509863</v>
       </c>
       <c r="J6" t="n">
         <v>100</v>
       </c>
       <c r="K6" t="n">
-        <v>3.895</v>
+        <v>3.938668</v>
       </c>
       <c r="L6" t="n">
-        <v>94.595</v>
+        <v>94.571196</v>
       </c>
       <c r="M6" t="n">
-        <v>98.48999999999999</v>
+        <v>98.509863</v>
       </c>
     </row>
     <row r="7">
@@ -1644,37 +1644,37 @@
         <v>360</v>
       </c>
       <c r="C7" t="n">
-        <v>8.497773</v>
+        <v>8.531285</v>
       </c>
       <c r="D7" t="n">
-        <v>1.592282</v>
+        <v>1.53222</v>
       </c>
       <c r="E7" t="n">
-        <v>2.535362</v>
+        <v>2.347697</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>8.108155</v>
+        <v>8.099916</v>
       </c>
       <c r="H7" t="n">
-        <v>8.953448</v>
+        <v>8.950123</v>
       </c>
       <c r="I7" t="n">
-        <v>9.471474000000001</v>
+        <v>9.478452000000001</v>
       </c>
       <c r="J7" t="n">
         <v>10</v>
       </c>
       <c r="K7" t="n">
-        <v>1.363318</v>
+        <v>1.378535</v>
       </c>
       <c r="L7" t="n">
-        <v>8.108155</v>
+        <v>8.099916</v>
       </c>
       <c r="M7" t="n">
-        <v>9.471474000000001</v>
+        <v>9.478452000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1763,37 +1763,37 @@
         <v>360</v>
       </c>
       <c r="C2" t="n">
-        <v>3.46923</v>
+        <v>4.312451</v>
       </c>
       <c r="D2" t="n">
-        <v>1.445621</v>
+        <v>1.458158</v>
       </c>
       <c r="E2" t="n">
-        <v>2.08982</v>
+        <v>2.126226</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>2.695203</v>
+        <v>3.357733</v>
       </c>
       <c r="H2" t="n">
-        <v>3.414805</v>
+        <v>4.250709</v>
       </c>
       <c r="I2" t="n">
-        <v>4.173039</v>
+        <v>5.078103</v>
       </c>
       <c r="J2" t="n">
         <v>10</v>
       </c>
       <c r="K2" t="n">
-        <v>1.477836</v>
+        <v>1.72037</v>
       </c>
       <c r="L2" t="n">
-        <v>2.695203</v>
+        <v>3.357733</v>
       </c>
       <c r="M2" t="n">
-        <v>4.173039</v>
+        <v>5.078103</v>
       </c>
     </row>
     <row r="3">
@@ -1806,37 +1806,37 @@
         <v>360</v>
       </c>
       <c r="C3" t="n">
-        <v>0.510338</v>
+        <v>0.438089</v>
       </c>
       <c r="D3" t="n">
-        <v>0.077488</v>
+        <v>0.079605</v>
       </c>
       <c r="E3" t="n">
-        <v>0.006004</v>
+        <v>0.006337</v>
       </c>
       <c r="F3" t="n">
-        <v>0.324382</v>
+        <v>0.202659</v>
       </c>
       <c r="G3" t="n">
-        <v>0.468849</v>
+        <v>0.385968</v>
       </c>
       <c r="H3" t="n">
-        <v>0.507421</v>
+        <v>0.434719</v>
       </c>
       <c r="I3" t="n">
-        <v>0.548064</v>
+        <v>0.479889</v>
       </c>
       <c r="J3" t="n">
-        <v>0.860398</v>
+        <v>0.748591</v>
       </c>
       <c r="K3" t="n">
-        <v>0.07921400000000001</v>
+        <v>0.09392</v>
       </c>
       <c r="L3" t="n">
-        <v>0.468849</v>
+        <v>0.385968</v>
       </c>
       <c r="M3" t="n">
-        <v>0.548064</v>
+        <v>0.479889</v>
       </c>
     </row>
     <row r="4">
@@ -1849,37 +1849,37 @@
         <v>360</v>
       </c>
       <c r="C4" t="n">
-        <v>21942.194444</v>
+        <v>25720.75908</v>
       </c>
       <c r="D4" t="n">
-        <v>1896.302811</v>
+        <v>6344.697462</v>
       </c>
       <c r="E4" t="n">
-        <v>3595964.35108</v>
+        <v>40255185.883786</v>
       </c>
       <c r="F4" t="n">
-        <v>15600</v>
+        <v>12746.307692</v>
       </c>
       <c r="G4" t="n">
-        <v>21275</v>
+        <v>21462.886451</v>
       </c>
       <c r="H4" t="n">
-        <v>21460</v>
+        <v>24788.574272</v>
       </c>
       <c r="I4" t="n">
-        <v>23420</v>
+        <v>28218.407391</v>
       </c>
       <c r="J4" t="n">
-        <v>29320</v>
+        <v>56621.089041</v>
       </c>
       <c r="K4" t="n">
-        <v>2145</v>
+        <v>6755.52094</v>
       </c>
       <c r="L4" t="n">
-        <v>21275</v>
+        <v>21462.886451</v>
       </c>
       <c r="M4" t="n">
-        <v>23420</v>
+        <v>28218.407391</v>
       </c>
     </row>
     <row r="5">
@@ -1892,37 +1892,37 @@
         <v>360</v>
       </c>
       <c r="C5" t="n">
-        <v>4.622591</v>
+        <v>2.957155</v>
       </c>
       <c r="D5" t="n">
-        <v>1.382145</v>
+        <v>1.446092</v>
       </c>
       <c r="E5" t="n">
-        <v>1.910325</v>
+        <v>2.091182</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>4.136297</v>
+        <v>1.986695</v>
       </c>
       <c r="H5" t="n">
-        <v>4.271137</v>
+        <v>2.74469</v>
       </c>
       <c r="I5" t="n">
-        <v>5.699708</v>
+        <v>3.526422</v>
       </c>
       <c r="J5" t="n">
         <v>10</v>
       </c>
       <c r="K5" t="n">
-        <v>1.563411</v>
+        <v>1.539728</v>
       </c>
       <c r="L5" t="n">
-        <v>4.136297</v>
+        <v>1.986695</v>
       </c>
       <c r="M5" t="n">
-        <v>5.699708</v>
+        <v>3.526422</v>
       </c>
     </row>
     <row r="6">
@@ -1935,37 +1935,37 @@
         <v>360</v>
       </c>
       <c r="C6" t="n">
-        <v>0.791124</v>
+        <v>0.701325</v>
       </c>
       <c r="D6" t="n">
-        <v>0.06003</v>
+        <v>0.089285</v>
       </c>
       <c r="E6" t="n">
-        <v>0.003604</v>
+        <v>0.007972</v>
       </c>
       <c r="F6" t="n">
-        <v>0.5270860000000001</v>
+        <v>0.303152</v>
       </c>
       <c r="G6" t="n">
-        <v>0.761711</v>
+        <v>0.657126</v>
       </c>
       <c r="H6" t="n">
-        <v>0.799942</v>
+        <v>0.7153389999999999</v>
       </c>
       <c r="I6" t="n">
-        <v>0.834028</v>
+        <v>0.761906</v>
       </c>
       <c r="J6" t="n">
-        <v>0.9028389999999999</v>
+        <v>0.877892</v>
       </c>
       <c r="K6" t="n">
-        <v>0.07231700000000001</v>
+        <v>0.104781</v>
       </c>
       <c r="L6" t="n">
-        <v>0.761711</v>
+        <v>0.657126</v>
       </c>
       <c r="M6" t="n">
-        <v>0.834028</v>
+        <v>0.761906</v>
       </c>
     </row>
     <row r="7">
@@ -1978,37 +1978,37 @@
         <v>360</v>
       </c>
       <c r="C7" t="n">
-        <v>7.026902</v>
+        <v>6.92788</v>
       </c>
       <c r="D7" t="n">
-        <v>1.597605</v>
+        <v>1.553492</v>
       </c>
       <c r="E7" t="n">
-        <v>2.552343</v>
+        <v>2.413337</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>6.244137</v>
+        <v>6.15885</v>
       </c>
       <c r="H7" t="n">
-        <v>7.261579</v>
+        <v>7.171719</v>
       </c>
       <c r="I7" t="n">
-        <v>8.168734000000001</v>
+        <v>7.981949</v>
       </c>
       <c r="J7" t="n">
         <v>10</v>
       </c>
       <c r="K7" t="n">
-        <v>1.924598</v>
+        <v>1.823098</v>
       </c>
       <c r="L7" t="n">
-        <v>6.244137</v>
+        <v>6.15885</v>
       </c>
       <c r="M7" t="n">
-        <v>8.168734000000001</v>
+        <v>7.981949</v>
       </c>
     </row>
     <row r="8">
@@ -2021,37 +2021,37 @@
         <v>360</v>
       </c>
       <c r="C8" t="n">
-        <v>0.857777</v>
+        <v>0.8608710000000001</v>
       </c>
       <c r="D8" t="n">
-        <v>0.07058399999999999</v>
+        <v>0.062815</v>
       </c>
       <c r="E8" t="n">
-        <v>0.004982</v>
+        <v>0.003946</v>
       </c>
       <c r="F8" t="n">
-        <v>0.3575</v>
+        <v>0.583333</v>
       </c>
       <c r="G8" t="n">
-        <v>0.822188</v>
+        <v>0.829693</v>
       </c>
       <c r="H8" t="n">
-        <v>0.8700599999999999</v>
+        <v>0.8657280000000001</v>
       </c>
       <c r="I8" t="n">
-        <v>0.898423</v>
+        <v>0.9</v>
       </c>
       <c r="J8" t="n">
         <v>1</v>
       </c>
       <c r="K8" t="n">
-        <v>0.076236</v>
+        <v>0.07030699999999999</v>
       </c>
       <c r="L8" t="n">
-        <v>0.822188</v>
+        <v>0.829693</v>
       </c>
       <c r="M8" t="n">
-        <v>0.898423</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="9">
@@ -2064,37 +2064,37 @@
         <v>360</v>
       </c>
       <c r="C9" t="n">
-        <v>7.786414</v>
+        <v>6.660911</v>
       </c>
       <c r="D9" t="n">
-        <v>1.098588</v>
+        <v>1.507564</v>
       </c>
       <c r="E9" t="n">
-        <v>1.206896</v>
+        <v>2.272749</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>7.23249</v>
+        <v>5.912642</v>
       </c>
       <c r="H9" t="n">
-        <v>7.977588</v>
+        <v>6.777463</v>
       </c>
       <c r="I9" t="n">
-        <v>8.419041999999999</v>
+        <v>7.599998</v>
       </c>
       <c r="J9" t="n">
         <v>10</v>
       </c>
       <c r="K9" t="n">
-        <v>1.186551</v>
+        <v>1.687356</v>
       </c>
       <c r="L9" t="n">
-        <v>7.23249</v>
+        <v>5.912642</v>
       </c>
       <c r="M9" t="n">
-        <v>8.419041999999999</v>
+        <v>7.599998</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
feat: L'Île-Rousse ajoutée aux réseaux de bus urbains d'Opp3 (A Balanina, depuis mai 2022, transport.data.gouv.fr) ; chaîne régénérée
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/stats_descriptives_betti_0_10.xlsx
+++ b/downloads/stats_descriptives_betti_0_10.xlsx
@@ -503,37 +503,37 @@
         <v>360</v>
       </c>
       <c r="C2" t="n">
-        <v>4.280791</v>
+        <v>4.280915</v>
       </c>
       <c r="D2" t="n">
-        <v>1.884743</v>
+        <v>1.881056</v>
       </c>
       <c r="E2" t="n">
-        <v>3.552256</v>
+        <v>3.538373</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>2.947068</v>
+        <v>2.957998</v>
       </c>
       <c r="H2" t="n">
-        <v>4.226464</v>
+        <v>4.22242</v>
       </c>
       <c r="I2" t="n">
-        <v>5.402328</v>
+        <v>5.398209</v>
       </c>
       <c r="J2" t="n">
         <v>10</v>
       </c>
       <c r="K2" t="n">
-        <v>2.45526</v>
+        <v>2.440211</v>
       </c>
       <c r="L2" t="n">
-        <v>2.947068</v>
+        <v>2.957998</v>
       </c>
       <c r="M2" t="n">
-        <v>5.402328</v>
+        <v>5.398209</v>
       </c>
     </row>
     <row r="3">
@@ -546,37 +546,37 @@
         <v>360</v>
       </c>
       <c r="C3" t="n">
-        <v>0.07385700000000001</v>
+        <v>0.073739</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0214</v>
+        <v>0.021362</v>
       </c>
       <c r="E3" t="n">
-        <v>0.000458</v>
+        <v>0.000456</v>
       </c>
       <c r="F3" t="n">
-        <v>0.025252</v>
+        <v>0.025123</v>
       </c>
       <c r="G3" t="n">
-        <v>0.058713</v>
+        <v>0.058715</v>
       </c>
       <c r="H3" t="n">
-        <v>0.07324</v>
+        <v>0.073074</v>
       </c>
       <c r="I3" t="n">
-        <v>0.086591</v>
+        <v>0.086427</v>
       </c>
       <c r="J3" t="n">
-        <v>0.138794</v>
+        <v>0.138686</v>
       </c>
       <c r="K3" t="n">
-        <v>0.027878</v>
+        <v>0.027712</v>
       </c>
       <c r="L3" t="n">
-        <v>0.058713</v>
+        <v>0.058715</v>
       </c>
       <c r="M3" t="n">
-        <v>0.086591</v>
+        <v>0.086427</v>
       </c>
     </row>
     <row r="4">
@@ -589,13 +589,13 @@
         <v>360</v>
       </c>
       <c r="C4" t="n">
-        <v>5.638079</v>
+        <v>5.64326</v>
       </c>
       <c r="D4" t="n">
-        <v>2.104138</v>
+        <v>2.108479</v>
       </c>
       <c r="E4" t="n">
-        <v>4.427398</v>
+        <v>4.445683</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -607,19 +607,19 @@
         <v>5.968596</v>
       </c>
       <c r="I4" t="n">
-        <v>7.419413</v>
+        <v>7.44575</v>
       </c>
       <c r="J4" t="n">
         <v>10</v>
       </c>
       <c r="K4" t="n">
-        <v>3.391255</v>
+        <v>3.417591</v>
       </c>
       <c r="L4" t="n">
         <v>4.028159</v>
       </c>
       <c r="M4" t="n">
-        <v>7.419413</v>
+        <v>7.44575</v>
       </c>
     </row>
     <row r="5">
@@ -632,13 +632,13 @@
         <v>360</v>
       </c>
       <c r="C5" t="n">
-        <v>0.424992</v>
+        <v>0.425293</v>
       </c>
       <c r="D5" t="n">
-        <v>0.122292</v>
+        <v>0.122544</v>
       </c>
       <c r="E5" t="n">
-        <v>0.014955</v>
+        <v>0.015017</v>
       </c>
       <c r="F5" t="n">
         <v>0.09730900000000001</v>
@@ -650,19 +650,19 @@
         <v>0.444201</v>
       </c>
       <c r="I5" t="n">
-        <v>0.528522</v>
+        <v>0.530053</v>
       </c>
       <c r="J5" t="n">
         <v>0.678505</v>
       </c>
       <c r="K5" t="n">
-        <v>0.197098</v>
+        <v>0.198629</v>
       </c>
       <c r="L5" t="n">
         <v>0.331424</v>
       </c>
       <c r="M5" t="n">
-        <v>0.528522</v>
+        <v>0.530053</v>
       </c>
     </row>
     <row r="6">
@@ -923,13 +923,13 @@
         <v>360</v>
       </c>
       <c r="C2" t="n">
-        <v>5.638079</v>
+        <v>5.64326</v>
       </c>
       <c r="D2" t="n">
-        <v>2.104138</v>
+        <v>2.108479</v>
       </c>
       <c r="E2" t="n">
-        <v>4.427398</v>
+        <v>4.445683</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -941,19 +941,19 @@
         <v>5.968596</v>
       </c>
       <c r="I2" t="n">
-        <v>7.419413</v>
+        <v>7.44575</v>
       </c>
       <c r="J2" t="n">
         <v>10</v>
       </c>
       <c r="K2" t="n">
-        <v>3.391255</v>
+        <v>3.417591</v>
       </c>
       <c r="L2" t="n">
         <v>4.028159</v>
       </c>
       <c r="M2" t="n">
-        <v>7.419413</v>
+        <v>7.44575</v>
       </c>
     </row>
     <row r="3">
@@ -966,13 +966,13 @@
         <v>360</v>
       </c>
       <c r="C3" t="n">
-        <v>0.424992</v>
+        <v>0.425293</v>
       </c>
       <c r="D3" t="n">
-        <v>0.122292</v>
+        <v>0.122544</v>
       </c>
       <c r="E3" t="n">
-        <v>0.014955</v>
+        <v>0.015017</v>
       </c>
       <c r="F3" t="n">
         <v>0.09730900000000001</v>
@@ -984,19 +984,19 @@
         <v>0.444201</v>
       </c>
       <c r="I3" t="n">
-        <v>0.528522</v>
+        <v>0.530053</v>
       </c>
       <c r="J3" t="n">
         <v>0.678505</v>
       </c>
       <c r="K3" t="n">
-        <v>0.197098</v>
+        <v>0.198629</v>
       </c>
       <c r="L3" t="n">
         <v>0.331424</v>
       </c>
       <c r="M3" t="n">
-        <v>0.528522</v>
+        <v>0.530053</v>
       </c>
     </row>
     <row r="4">
@@ -1181,13 +1181,13 @@
         <v>360</v>
       </c>
       <c r="C8" t="n">
-        <v>140.668614</v>
+        <v>140.946391</v>
       </c>
       <c r="D8" t="n">
-        <v>53.036811</v>
+        <v>53.503683</v>
       </c>
       <c r="E8" t="n">
-        <v>2812.903366</v>
+        <v>2862.644091</v>
       </c>
       <c r="F8" t="n">
         <v>63.636379</v>
@@ -1199,19 +1199,19 @@
         <v>173.055557</v>
       </c>
       <c r="I8" t="n">
-        <v>191.962104</v>
+        <v>192.001889</v>
       </c>
       <c r="J8" t="n">
         <v>294.288572</v>
       </c>
       <c r="K8" t="n">
-        <v>102.51731</v>
+        <v>102.557095</v>
       </c>
       <c r="L8" t="n">
         <v>89.444795</v>
       </c>
       <c r="M8" t="n">
-        <v>191.962104</v>
+        <v>192.001889</v>
       </c>
     </row>
     <row r="9">
@@ -1224,13 +1224,13 @@
         <v>360</v>
       </c>
       <c r="C9" t="n">
-        <v>3.339757</v>
+        <v>3.3518</v>
       </c>
       <c r="D9" t="n">
-        <v>2.299428</v>
+        <v>2.319669</v>
       </c>
       <c r="E9" t="n">
-        <v>5.287369</v>
+        <v>5.380866</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -1242,19 +1242,19 @@
         <v>4.743904</v>
       </c>
       <c r="I9" t="n">
-        <v>5.563603</v>
+        <v>5.565328</v>
       </c>
       <c r="J9" t="n">
         <v>10</v>
       </c>
       <c r="K9" t="n">
-        <v>4.444671</v>
+        <v>4.446396</v>
       </c>
       <c r="L9" t="n">
         <v>1.118932</v>
       </c>
       <c r="M9" t="n">
-        <v>5.563603</v>
+        <v>5.565328</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
feat(opp2): sens retourné (plus diversifié = mieux) et diversité de jour (actifs à leur commune de travail + retraités) ; mêmes données que visu_corse_simple ; tests
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/stats_descriptives_betti_0_10.xlsx
+++ b/downloads/stats_descriptives_betti_0_10.xlsx
@@ -503,37 +503,37 @@
         <v>360</v>
       </c>
       <c r="C2" t="n">
-        <v>4.280915</v>
+        <v>4.374485</v>
       </c>
       <c r="D2" t="n">
-        <v>1.881056</v>
+        <v>1.80521</v>
       </c>
       <c r="E2" t="n">
-        <v>3.538373</v>
+        <v>3.258782</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>2.957998</v>
+        <v>2.991409</v>
       </c>
       <c r="H2" t="n">
-        <v>4.22242</v>
+        <v>4.258347</v>
       </c>
       <c r="I2" t="n">
-        <v>5.398209</v>
+        <v>5.674786</v>
       </c>
       <c r="J2" t="n">
         <v>10</v>
       </c>
       <c r="K2" t="n">
-        <v>2.440211</v>
+        <v>2.683378</v>
       </c>
       <c r="L2" t="n">
-        <v>2.957998</v>
+        <v>2.991409</v>
       </c>
       <c r="M2" t="n">
-        <v>5.398209</v>
+        <v>5.674786</v>
       </c>
     </row>
     <row r="3">
@@ -546,37 +546,37 @@
         <v>360</v>
       </c>
       <c r="C3" t="n">
-        <v>0.073739</v>
+        <v>0.094068</v>
       </c>
       <c r="D3" t="n">
-        <v>0.021362</v>
+        <v>0.030649</v>
       </c>
       <c r="E3" t="n">
-        <v>0.000456</v>
+        <v>0.0009389999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>0.025123</v>
+        <v>0.019799</v>
       </c>
       <c r="G3" t="n">
-        <v>0.058715</v>
+        <v>0.070586</v>
       </c>
       <c r="H3" t="n">
-        <v>0.073074</v>
+        <v>0.092096</v>
       </c>
       <c r="I3" t="n">
-        <v>0.086427</v>
+        <v>0.116145</v>
       </c>
       <c r="J3" t="n">
-        <v>0.138686</v>
+        <v>0.189578</v>
       </c>
       <c r="K3" t="n">
-        <v>0.027712</v>
+        <v>0.045558</v>
       </c>
       <c r="L3" t="n">
-        <v>0.058715</v>
+        <v>0.070586</v>
       </c>
       <c r="M3" t="n">
-        <v>0.086427</v>
+        <v>0.116145</v>
       </c>
     </row>
     <row r="4">
@@ -589,37 +589,37 @@
         <v>360</v>
       </c>
       <c r="C4" t="n">
-        <v>5.64326</v>
+        <v>6.058121</v>
       </c>
       <c r="D4" t="n">
-        <v>2.108479</v>
+        <v>1.926101</v>
       </c>
       <c r="E4" t="n">
-        <v>4.445683</v>
+        <v>3.709865</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>4.028159</v>
+        <v>4.596022</v>
       </c>
       <c r="H4" t="n">
-        <v>5.968596</v>
+        <v>6.332201</v>
       </c>
       <c r="I4" t="n">
-        <v>7.44575</v>
+        <v>7.764058</v>
       </c>
       <c r="J4" t="n">
         <v>10</v>
       </c>
       <c r="K4" t="n">
-        <v>3.417591</v>
+        <v>3.168036</v>
       </c>
       <c r="L4" t="n">
-        <v>4.028159</v>
+        <v>4.596022</v>
       </c>
       <c r="M4" t="n">
-        <v>7.44575</v>
+        <v>7.764058</v>
       </c>
     </row>
     <row r="5">
@@ -632,37 +632,37 @@
         <v>360</v>
       </c>
       <c r="C5" t="n">
-        <v>0.425293</v>
+        <v>0.550644</v>
       </c>
       <c r="D5" t="n">
-        <v>0.122544</v>
+        <v>0.159705</v>
       </c>
       <c r="E5" t="n">
-        <v>0.015017</v>
+        <v>0.025506</v>
       </c>
       <c r="F5" t="n">
-        <v>0.09730900000000001</v>
+        <v>0.048329</v>
       </c>
       <c r="G5" t="n">
-        <v>0.331424</v>
+        <v>0.429413</v>
       </c>
       <c r="H5" t="n">
-        <v>0.444201</v>
+        <v>0.57337</v>
       </c>
       <c r="I5" t="n">
-        <v>0.530053</v>
+        <v>0.692094</v>
       </c>
       <c r="J5" t="n">
-        <v>0.678505</v>
+        <v>0.877489</v>
       </c>
       <c r="K5" t="n">
-        <v>0.198629</v>
+        <v>0.262681</v>
       </c>
       <c r="L5" t="n">
-        <v>0.331424</v>
+        <v>0.429413</v>
       </c>
       <c r="M5" t="n">
-        <v>0.530053</v>
+        <v>0.692094</v>
       </c>
     </row>
     <row r="6">
@@ -923,37 +923,37 @@
         <v>360</v>
       </c>
       <c r="C2" t="n">
-        <v>5.64326</v>
+        <v>6.058121</v>
       </c>
       <c r="D2" t="n">
-        <v>2.108479</v>
+        <v>1.926101</v>
       </c>
       <c r="E2" t="n">
-        <v>4.445683</v>
+        <v>3.709865</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>4.028159</v>
+        <v>4.596022</v>
       </c>
       <c r="H2" t="n">
-        <v>5.968596</v>
+        <v>6.332201</v>
       </c>
       <c r="I2" t="n">
-        <v>7.44575</v>
+        <v>7.764058</v>
       </c>
       <c r="J2" t="n">
         <v>10</v>
       </c>
       <c r="K2" t="n">
-        <v>3.417591</v>
+        <v>3.168036</v>
       </c>
       <c r="L2" t="n">
-        <v>4.028159</v>
+        <v>4.596022</v>
       </c>
       <c r="M2" t="n">
-        <v>7.44575</v>
+        <v>7.764058</v>
       </c>
     </row>
     <row r="3">
@@ -966,37 +966,37 @@
         <v>360</v>
       </c>
       <c r="C3" t="n">
-        <v>0.425293</v>
+        <v>0.550644</v>
       </c>
       <c r="D3" t="n">
-        <v>0.122544</v>
+        <v>0.159705</v>
       </c>
       <c r="E3" t="n">
-        <v>0.015017</v>
+        <v>0.025506</v>
       </c>
       <c r="F3" t="n">
-        <v>0.09730900000000001</v>
+        <v>0.048329</v>
       </c>
       <c r="G3" t="n">
-        <v>0.331424</v>
+        <v>0.429413</v>
       </c>
       <c r="H3" t="n">
-        <v>0.444201</v>
+        <v>0.57337</v>
       </c>
       <c r="I3" t="n">
-        <v>0.530053</v>
+        <v>0.692094</v>
       </c>
       <c r="J3" t="n">
-        <v>0.678505</v>
+        <v>0.877489</v>
       </c>
       <c r="K3" t="n">
-        <v>0.198629</v>
+        <v>0.262681</v>
       </c>
       <c r="L3" t="n">
-        <v>0.331424</v>
+        <v>0.429413</v>
       </c>
       <c r="M3" t="n">
-        <v>0.530053</v>
+        <v>0.692094</v>
       </c>
     </row>
     <row r="4">
@@ -1095,37 +1095,37 @@
         <v>360</v>
       </c>
       <c r="C6" t="n">
-        <v>0.389002</v>
+        <v>0.696013</v>
       </c>
       <c r="D6" t="n">
-        <v>0.19685</v>
+        <v>0.134877</v>
       </c>
       <c r="E6" t="n">
-        <v>0.03875</v>
+        <v>0.018192</v>
       </c>
       <c r="F6" t="n">
-        <v>0.120463</v>
+        <v>0.191472</v>
       </c>
       <c r="G6" t="n">
-        <v>0.259543</v>
+        <v>0.6157010000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>0.335847</v>
+        <v>0.717982</v>
       </c>
       <c r="I6" t="n">
-        <v>0.47874</v>
+        <v>0.795458</v>
       </c>
       <c r="J6" t="n">
-        <v>1.436583</v>
+        <v>0.906684</v>
       </c>
       <c r="K6" t="n">
-        <v>0.219197</v>
+        <v>0.179756</v>
       </c>
       <c r="L6" t="n">
-        <v>0.259543</v>
+        <v>0.6157010000000001</v>
       </c>
       <c r="M6" t="n">
-        <v>0.47874</v>
+        <v>0.795458</v>
       </c>
     </row>
     <row r="7">
@@ -1138,37 +1138,37 @@
         <v>360</v>
       </c>
       <c r="C7" t="n">
-        <v>2.040383</v>
+        <v>7.054428</v>
       </c>
       <c r="D7" t="n">
-        <v>1.495682</v>
+        <v>1.885837</v>
       </c>
       <c r="E7" t="n">
-        <v>2.237064</v>
+        <v>3.556382</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>1.056743</v>
+        <v>5.931513</v>
       </c>
       <c r="H7" t="n">
-        <v>1.636503</v>
+        <v>7.361589</v>
       </c>
       <c r="I7" t="n">
-        <v>2.72222</v>
+        <v>8.444845000000001</v>
       </c>
       <c r="J7" t="n">
         <v>10</v>
       </c>
       <c r="K7" t="n">
-        <v>1.665477</v>
+        <v>2.513332</v>
       </c>
       <c r="L7" t="n">
-        <v>1.056743</v>
+        <v>5.931513</v>
       </c>
       <c r="M7" t="n">
-        <v>2.72222</v>
+        <v>8.444845000000001</v>
       </c>
     </row>
     <row r="8">

</xml_diff>